<commit_message>
feat(securite+benin+perf): RLS approfondie prouvée par attaques (OrThrow, organization, garde FK étrangère, portée enfant ledgerline, runWithRls étanche) — 28/28 ; Country Pack Bénin v1.1.0 (IFU dérivé du pack dans exports SYSCOHADA, seed BJ équilibré 23,07 M XOF, INV-011 matrice) ; tests de charge exports (11k écritures/29k lignes, p95 HTTP 1,16 s, 0 erreur) ; régressions 63+32+22+24+6 vertes, tsc/eslint clean
</commit_message>
<xml_diff>
--- a/scripts/out_syscohada/balance_bj.xlsx
+++ b/scripts/out_syscohada/balance_bj.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="41">
   <si>
     <t>YAHRIA BUSINESS OS — ÉTATS FINANCIERS SYSCOHADA (SYSTÈME NORMAL)</t>
   </si>
   <si>
-    <t>GOLFE TRADING &amp; SERVICES SARL · NCC 3202411456789 · RCCM RB/COT/23 A 14567 · BJ · Monnaie : XOF</t>
+    <t>GOLFE TRADING &amp; SERVICES SARL · IFU 3202411456789 · RCCM RB/COT/23 A 14567 · BJ · Monnaie : XOF</t>
   </si>
   <si>
     <t>BALANCE GÉNÉRALE DES COMPTES — Période : 01/01/2026 — 31/12/2026</t>
@@ -88,12 +88,30 @@
     <t>CLASSE 6 — Comptes de charges</t>
   </si>
   <si>
+    <t>601</t>
+  </si>
+  <si>
+    <t>Achats de matières premières</t>
+  </si>
+  <si>
+    <t>61</t>
+  </si>
+  <si>
+    <t>Transports</t>
+  </si>
+  <si>
     <t>622</t>
   </si>
   <si>
     <t>Locations et charges locatives</t>
   </si>
   <si>
+    <t>628</t>
+  </si>
+  <si>
+    <t>Frais de télécommunications</t>
+  </si>
+  <si>
     <t>CLASSE 7 — Comptes de produits</t>
   </si>
   <si>
@@ -101,6 +119,12 @@
   </si>
   <si>
     <t>Ventes de produits finis</t>
+  </si>
+  <si>
+    <t>706</t>
+  </si>
+  <si>
+    <t>Prestations de services</t>
   </si>
   <si>
     <t>TOTAUX</t>
@@ -566,7 +590,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -653,16 +677,16 @@
         <v>4</v>
       </c>
       <c r="D7" s="6">
-        <v>200000</v>
+        <v>3141400</v>
       </c>
       <c r="E7" s="6">
-        <v>0</v>
+        <v>3501900</v>
       </c>
       <c r="F7" s="6">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="G7" s="6">
-        <v>0</v>
+        <v>360500</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -676,13 +700,13 @@
         <v>4</v>
       </c>
       <c r="D8" s="6">
-        <v>2416050</v>
+        <v>9924390</v>
       </c>
       <c r="E8" s="6">
-        <v>811250</v>
+        <v>5499390</v>
       </c>
       <c r="F8" s="6">
-        <v>1604800</v>
+        <v>4425000</v>
       </c>
       <c r="G8" s="6">
         <v>0</v>
@@ -702,13 +726,13 @@
         <v>0</v>
       </c>
       <c r="E9" s="6">
-        <v>368550</v>
+        <v>1513890</v>
       </c>
       <c r="F9" s="6">
         <v>0</v>
       </c>
       <c r="G9" s="6">
-        <v>368550</v>
+        <v>1513890</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -722,13 +746,13 @@
         <v>4</v>
       </c>
       <c r="D10" s="6">
-        <v>153000</v>
+        <v>549900</v>
       </c>
       <c r="E10" s="6">
         <v>0</v>
       </c>
       <c r="F10" s="6">
-        <v>153000</v>
+        <v>549900</v>
       </c>
       <c r="G10" s="6">
         <v>0</v>
@@ -756,16 +780,16 @@
         <v>5</v>
       </c>
       <c r="D12" s="6">
-        <v>0</v>
+        <v>2655000</v>
       </c>
       <c r="E12" s="6">
-        <v>1203000</v>
+        <v>3578000</v>
       </c>
       <c r="F12" s="6">
         <v>0</v>
       </c>
       <c r="G12" s="6">
-        <v>1203000</v>
+        <v>923000</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -779,13 +803,13 @@
         <v>5</v>
       </c>
       <c r="D13" s="6">
-        <v>811250</v>
+        <v>2844390</v>
       </c>
       <c r="E13" s="6">
-        <v>0</v>
+        <v>566400</v>
       </c>
       <c r="F13" s="6">
-        <v>811250</v>
+        <v>2277990</v>
       </c>
       <c r="G13" s="6">
         <v>0</v>
@@ -813,78 +837,170 @@
         <v>6</v>
       </c>
       <c r="D15" s="6">
-        <v>850000</v>
+        <v>1250000</v>
       </c>
       <c r="E15" s="6">
         <v>0</v>
       </c>
       <c r="F15" s="6">
-        <v>850000</v>
+        <v>1250000</v>
       </c>
       <c r="G15" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
+      <c r="A16" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16">
+        <v>6</v>
+      </c>
+      <c r="D16" s="6">
+        <v>790000</v>
+      </c>
+      <c r="E16" s="6">
+        <v>0</v>
+      </c>
+      <c r="F16" s="6">
+        <v>790000</v>
+      </c>
+      <c r="G16" s="6">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C17">
+        <v>6</v>
+      </c>
+      <c r="D17" s="6">
+        <v>1750000</v>
+      </c>
+      <c r="E17" s="6">
+        <v>0</v>
+      </c>
+      <c r="F17" s="6">
+        <v>1750000</v>
+      </c>
+      <c r="G17" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18">
+        <v>6</v>
+      </c>
+      <c r="D18" s="6">
+        <v>165000</v>
+      </c>
+      <c r="E18" s="6">
+        <v>0</v>
+      </c>
+      <c r="F18" s="6">
+        <v>165000</v>
+      </c>
+      <c r="G18" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20">
         <v>7</v>
       </c>
-      <c r="D17" s="6">
-        <v>0</v>
-      </c>
-      <c r="E17" s="6">
-        <v>2047500</v>
-      </c>
-      <c r="F17" s="6">
-        <v>0</v>
-      </c>
-      <c r="G17" s="6">
-        <v>2047500</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="9">
-        <v>4430300</v>
-      </c>
-      <c r="E18" s="9">
-        <v>4430300</v>
-      </c>
-      <c r="F18" s="9">
-        <v>3619050</v>
-      </c>
-      <c r="G18" s="9">
-        <v>3619050</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
-        <v>32</v>
+      <c r="D20" s="6">
+        <v>0</v>
+      </c>
+      <c r="E20" s="6">
+        <v>6160500</v>
+      </c>
+      <c r="F20" s="6">
+        <v>0</v>
+      </c>
+      <c r="G20" s="6">
+        <v>6160500</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21">
+        <v>7</v>
+      </c>
+      <c r="D21" s="6">
+        <v>0</v>
+      </c>
+      <c r="E21" s="6">
+        <v>2250000</v>
+      </c>
+      <c r="F21" s="6">
+        <v>0</v>
+      </c>
+      <c r="G21" s="6">
+        <v>2250000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" s="9">
+        <v>23070080</v>
+      </c>
+      <c r="E22" s="9">
+        <v>23070080</v>
+      </c>
+      <c r="F22" s="9">
+        <v>11207890</v>
+      </c>
+      <c r="G22" s="9">
+        <v>11207890</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +1011,7 @@
     <mergeCell ref="A6:G6"/>
     <mergeCell ref="A11:G11"/>
     <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A19:G19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>